<commit_message>
feat(security): Expand security suite to 300 comprehensive test cases across 10 cybersecurity domains
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/endpoint-inventory.xlsx
+++ b/Vulnerability Test Results/endpoint-inventory.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,24 +40,6 @@
     <font>
       <name val="Calibri"/>
       <color rgb="001E293B"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00059669"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="002563EB"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00DC2626"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -113,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -122,29 +104,11 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -512,15 +476,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="39" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -573,7 +537,7 @@
           <t>GET</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -595,32 +559,32 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>/api/auth/user/{user_id}</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Self / Admin</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>backend/app/api/auth.py:25</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Get single user account profile</t>
         </is>
@@ -632,12 +596,12 @@
           <t>/api/auth/register</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -659,32 +623,32 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>/api/auth/login</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Public / All</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>backend/app/api/auth.py:82</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Authenticate user via username/email &amp; password</t>
         </is>
@@ -701,7 +665,7 @@
           <t>GET</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>No (Query user_id)</t>
         </is>
@@ -723,32 +687,32 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>/api/auth/reset-progress</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>No (Body user_id)</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Self / User</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>backend/app/api/auth.py:180</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Reset concept mastery and quiz attempts</t>
         </is>
@@ -760,12 +724,12 @@
           <t>/api/auth/send-otp</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -787,32 +751,32 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>/api/auth/verify-otp</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Public / All</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>backend/app/api/auth.py:270</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Verify 6-digit OTP code and authenticate</t>
         </is>
@@ -829,7 +793,7 @@
           <t>GET</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -851,32 +815,32 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>/api/courses/{course_id}</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Public / Student</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>backend/app/api/courses.py:35</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Get details and stats for a specific course</t>
         </is>
@@ -888,12 +852,12 @@
           <t>/api/courses</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -915,32 +879,32 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>/api/courses/generate-with-ai</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Authenticated</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>backend/app/api/courses.py:101</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Synthesize dynamic topic DAG curriculum</t>
         </is>
@@ -952,12 +916,12 @@
           <t>/api/courses/seed-all</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -979,32 +943,32 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>/api/courses/{course_id}</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Instructor / Admin</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>backend/app/api/courses.py:220</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>Delete course and associated concept nodes</t>
         </is>
@@ -1021,7 +985,7 @@
           <t>GET</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1043,32 +1007,32 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>/api/concepts/{concept_id}/deep-briefing</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>Student / All</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>backend/app/api/concepts.py:54</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>Exhaustive deep conceptual briefing</t>
         </is>
@@ -1085,7 +1049,7 @@
           <t>GET</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>No (Query user_id)</t>
         </is>
@@ -1107,169 +1071,169 @@
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>/api/concepts</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>Instructor</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>backend/app/api/concepts.py:175</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>Create new concept node in course</t>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>/api/learning-paths/generate</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>No (Query target_concept_id)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Student / All</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>backend/app/api/learning_paths.py:16</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Generate optimal prerequisite learning sequence</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>/api/concepts/dependency</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
+          <t>/api/learning-paths/bottlenecks</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Instructor</t>
+          <t>Instructor / Admin</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>backend/app/api/concepts.py:210</t>
+          <t>backend/app/api/learning_paths.py:48</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Link prerequisite dependency edge between nodes</t>
+          <t>Identify critical learning graph bottlenecks</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>/api/concepts/{concept_id}</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>DELETE</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>Instructor</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>backend/app/api/concepts.py:250</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>Remove concept node and downstream edges</t>
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>/api/quiz/concept/{concept_id}</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Student / All</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>backend/app/api/quiz.py:16</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Generate 20-question diagnostic micro-quiz</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>/api/concepts/dependency/{dep_id}</t>
-        </is>
-      </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>DELETE</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>/api/quiz/submit</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>No (Body user_id)</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Instructor</t>
+          <t>Student / Self</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>backend/app/api/concepts.py:280</t>
+          <t>backend/app/api/quiz.py:65</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Remove prerequisite dependency relationship</t>
+          <t>Evaluate student quiz responses &amp; update mastery</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>/api/concepts/sync-firebase</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>backend/app/api/concepts.py:310</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>Synchronize SQLite concepts to Firebase RTDB</t>
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>/api/analytics/overview</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Instructor / Admin</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>backend/app/api/analytics.py:14</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Aggregate institutional cohort mastery analytics</t>
         </is>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>/api/learning-paths/generate</t>
+          <t>/api/analytics/at-risk-students</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1277,63 +1241,63 @@
           <t>GET</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>No (Query params)</t>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>Instructor / Admin</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>backend/app/api/learning_paths.py:18</t>
+          <t>backend/app/api/analytics.py:42</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Compute optimal topological prerequisite sequence</t>
+          <t>Identify students at academic risk</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>/api/learning-paths/bottlenecks/{course_id}</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>Instructor / Researcher</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>backend/app/api/learning_paths.py:65</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>Identify critical prerequisite bottleneck nodes</t>
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>/docs</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Public (Swagger UI)</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>backend/main.py:16</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Interactive OpenAPI documentation interface</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>/api/quiz/concept/{concept_id}</t>
+          <t>/openapi.json</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -1341,312 +1305,24 @@
           <t>GET</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>Public</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>backend/app/api/quiz.py:21</t>
+          <t>backend/main.py:16</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Get or generate 20-question diagnostic quiz</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>/api/quiz</t>
-        </is>
-      </c>
-      <c r="B28" s="10" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>Instructor</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>backend/app/api/quiz.py:95</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>Create or overwrite custom assessment quiz</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>/api/quiz/submit</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>No (Body user_id)</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>Authenticated Student</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>backend/app/api/quiz.py:167</t>
-        </is>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>Submit diagnostic quiz attempt answers</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>/api/quiz/attempts/user/{user_id}</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>Self / Instructor</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>backend/app/api/quiz.py:260</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>Retrieve student historical quiz attempts</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>/api/analytics/comparative-study</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>Researcher / Instructor</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>backend/app/api/analytics.py:18</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>Comparative analytics Group A vs Group B</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>/api/analytics/concept-difficulty/{course_id}</t>
-        </is>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>Instructor</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>backend/app/api/analytics.py:75</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>Compute concept difficulty &amp; failure rates</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>/api/analytics/student-progress/{user_id}</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>Self / Instructor</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>backend/app/api/analytics.py:120</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>Detailed student learning progression breakdown</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>/api/ai-tutor/query</t>
-        </is>
-      </c>
-      <c r="B34" s="10" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>Student</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="inlineStr">
-        <is>
-          <t>backend/app/api/ai_tutor.py:20</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>Socratic AI Tutor conversational assistance</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>/api/ai-tutor/remediation-advice/{concept_id}</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>Student</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>backend/app/api/ai_tutor.py:65</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>Diagnostic remediation and mental model guidance</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>Public</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="inlineStr">
-        <is>
-          <t>backend/main.py:40</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>Root API operational status and service health</t>
+          <t>Machine-readable OpenAPI 3.0 schema definition</t>
         </is>
       </c>
     </row>

</xml_diff>